<commit_message>
Task tracker: the GPU is g5.2xlarge; dependencies checked at a022c2c
My tasks: L-09 and L-10 describe the A10G and g5.2xlarge (8 vCPUs a
job), not the L40S on g6e, which Sydney does not offer.

Waiting on others, checked again: the jobs framework's tests pass
against MySQL; the GPU quota is for Flex's AWS team, at 8 vCPUs a host;
where the nvdiffrast options are written up; and a row for the real AWS
account numbers, which the first image build needs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Tejesh-3D-Tasks.xlsx
+++ b/docs/Tejesh-3D-Tasks.xlsx
@@ -1414,7 +1414,7 @@
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Docker image built for the NVIDIA L40S (CUDA 12.4 build stage, slim runtime) in ECR; weights copied once into S3; stateless entry point: S3 frames in, GLB out. Replaces the RunPod kit.</t>
+          <t>Docker image built for the NVIDIA A10G and L4 (CUDA 12.4 build stage, slim runtime) in ECR; weights copied once into S3; stateless entry point: S3 frames in, GLB out. Replaces the RunPod kit.</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
@@ -1450,7 +1450,7 @@
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>AWS Batch on g6e.xlarge in Sydney, scaling to zero when idle; job definition; infrastructure code inside the backend's CDK app.</t>
+          <t>AWS Batch on g5.2xlarge in Sydney, scaling to zero when idle; job definition; infrastructure code inside the backend's CDK app.</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>Built: infra/lib/gpu-stack.ts (in each stage, between Data and Api, only when cdk.json names an approved image by digest): AWS Batch in Sydney on g6e.xlarge, min 0 vCPUs (scales to zero), max 4 x gpuMaxInstances (dev 1, staging 1, prod 2), Amazon Linux 2023 NVIDIA, private subnets; launch template mounting the host's NVMe at /weights (uid 1000) and a 100 GB encrypted root; job definition &lt;prefix&gt;-trellis2 (image by digest, 1 GPU, 4 vCPU, 28 GiB, /weights host volume, 1 h, 3 attempts, EXIT on code 2); job role scoped to the weights (read) and models/accounts/*/assets/* (read/write); execution role pulls cross-account from ECR; job outcomes via EventBridge to the gpu-jobs queue. Api stack: TRELLIS2_JOB_QUEUE/DEFINITION, batch:SubmitJob, gpu-jobs consume. Config refuses an image by tag. 17 infra tests pass.</t>
+          <t>Built: infra/lib/gpu-stack.ts (in each stage, between Data and Api, only when cdk.json names an approved image by digest): AWS Batch in Sydney on g5.2xlarge (g6e, the first choice, is not offered in Sydney), min 0 vCPUs (scales to zero), max 8 x gpuMaxInstances (dev 1, staging 1, prod 2), Amazon Linux 2023 NVIDIA, private subnets; launch template mounting the host's NVMe at /weights (uid 1000) and a 100 GB encrypted root; job definition &lt;prefix&gt;-trellis2 (image by digest, 1 GPU, 8 vCPU, 28 GiB, /weights host volume, 1 h, 3 attempts, EXIT on code 2); job role scoped to the weights (read) and models/accounts/*/assets/* (read/write); execution role pulls cross-account from ECR; job outcomes via EventBridge to the gpu-jobs queue. Api stack: TRELLIS2_JOB_QUEUE/DEFINITION, batch:SubmitJob, gpu-jobs consume. Config refuses an image by tag. 17 infra tests pass.</t>
         </is>
       </c>
     </row>
@@ -2317,7 +2317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2353,7 +2353,7 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Status (checked at 91c737d)</t>
+          <t>Status (checked at a022c2c)</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -2449,7 +2449,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>Built: backend/src/jobs (tests need MySQL; not run yet)</t>
+          <t>Built: backend/src/jobs; its tests pass against MySQL (backend suite, 299 passed)</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -2481,7 +2481,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Built (tests need MySQL; not run yet)</t>
+          <t>Built; its tests pass against MySQL (backend suite, 299 passed)</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -2732,12 +2732,12 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Thomas</t>
+          <t>Flex's AWS team</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>Not checked: an AWS account request</t>
+          <t>Not requested. Hosts are g5.2xlarge (8 vCPUs): ask for 16 in dev and staging, 32 in prod (docs/runbooks/service-quotas.md)</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -2769,7 +2769,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Not started. The options and their costs: docs/trellis2-before-deployment.md, sections 2 and 6</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
@@ -2812,6 +2812,38 @@
       <c r="F17" s="4" t="inlineStr">
         <is>
           <t>Request access on huggingface.co/facebook/dinov3-vitl16-pretrain-lvd1689m from the company's Hugging Face account; Meta approves by hand. Then run gpu/trellis2/lock_weights.py with that account's HF_TOKEN to lock DINOv3's hashes; until then fetch_weights.py refuses its files.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Accounts</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Real AWS account numbers in infra/cdk.json; the accounts bootstrapped; the pipelines and environments deployed</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Thomas, Flex's AWS team</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Placeholders in infra/cdk.json</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>L-09, L-10, L-14</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>The accounts the image pipeline builds in and the GPU environment deploys into: the first image build, the weights copy and the golden test all need them (docs/deployment-guide.md, 2.1 to 2.6).</t>
         </is>
       </c>
     </row>

</xml_diff>